<commit_message>
field-operations: required site location, photo filing and approval walkthrough
- Sites require a location; the label derives from it, the unit number is
  optional and part of duplicate identity; imports need coordinates for new sites.
- Photo evidence: create asks for the parent and the photo only; provenance is
  set by the server.
- Seed member mapping keeps optional phone/active without fabricating numbers.
- README/docs: full walkthrough with new real-UI captures — RFC/resubmit/approve,
  rejection restoring the amount, photo inspection facts, Controller site
  handover with four downloads, Envoy agent channel reconnected without QR.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/field-operations/tests/fixtures/job-import.xlsx
+++ b/field-operations/tests/fixtures/job-import.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -432,6 +432,9 @@
     <col width="44" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,11 +478,26 @@
           <t>external_ref</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t>unit_number</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t>latitude</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t>longitude</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Blk 412 Tampines Street 41 #07-221</t>
+          <t>Blk 412 Tampines Street 41</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -510,6 +528,17 @@
         <is>
           <t>IMP-1001</t>
         </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>#07-221</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>1.3572</v>
+      </c>
+      <c r="K2" t="n">
+        <v>103.9466</v>
       </c>
     </row>
     <row r="3">
@@ -547,6 +576,12 @@
           <t>IMP-1002</t>
         </is>
       </c>
+      <c r="J3" t="n">
+        <v>1.3572</v>
+      </c>
+      <c r="K3" t="n">
+        <v>103.9466</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -583,6 +618,12 @@
           <t>IMP-1003</t>
         </is>
       </c>
+      <c r="J4" t="n">
+        <v>1.3199</v>
+      </c>
+      <c r="K4" t="n">
+        <v>103.9167</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -611,6 +652,12 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
+      <c r="J5" t="n">
+        <v>1.2794</v>
+      </c>
+      <c r="K5" t="n">
+        <v>103.8536</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -646,6 +693,12 @@
         <is>
           <t>IMP-1005</t>
         </is>
+      </c>
+      <c r="J6" t="n">
+        <v>1.3273</v>
+      </c>
+      <c r="K6" t="n">
+        <v>103.9334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move templates to the layer-map model surface and Effect 4.0.6
Read and write declarations are layer maps; policies guard each model's access points with
per-layer columns and typed check callbacks; declared queries become page reads plus src/lib
helpers; writes are batches. Field operations drops variations, keeps job status to
pending/completed, links contractors by email or phone, notifies controllers of new suspicion
logs and gives the WhatsApp envoy an acknowledge-first recipe. Effect 4.0.6 and vitest 5.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/field-operations/tests/fixtures/job-import.xlsx
+++ b/field-operations/tests/fixtures/job-import.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Jobs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>assignee_user_id</t>
+          <t>assignee_contact</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -478,17 +478,17 @@
           <t>external_ref</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>unit_number</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="1">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>latitude</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>longitude</t>
         </is>
@@ -523,7 +523,6 @@
           <t>Site survey for window grille replacement.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>IMP-1001</t>
@@ -570,7 +569,6 @@
           <t>Install 4 window grilles per survey.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>IMP-1002</t>
@@ -612,7 +610,6 @@
           <t>Inspect roof leak above master bedroom.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>IMP-1003</t>
@@ -650,8 +647,6 @@
           <t>Service 6 FCUs on level 21.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
       <c r="J5" t="n">
         <v>1.2794</v>
       </c>
@@ -688,7 +683,6 @@
           <t>Final walkthrough and key handover.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>IMP-1005</t>

</xml_diff>